<commit_message>
dados: 2026-10-12 17:26 (132 arquivos)
</commit_message>
<xml_diff>
--- a/xlsx/carteira_mensal/Abr_2026.xlsx
+++ b/xlsx/carteira_mensal/Abr_2026.xlsx
@@ -75,22 +75,22 @@
     <t>Data de Criação do Projeto</t>
   </si>
   <si>
+    <t>/  /     até   /  /</t>
+  </si>
+  <si>
+    <t>Data de Criação do Orçamento</t>
+  </si>
+  <si>
+    <t>/  /     00:00 até   /  /     00:00</t>
+  </si>
+  <si>
+    <t>Data de Criação do Contrato</t>
+  </si>
+  <si>
+    <t>Data de Assinatura do Contrato</t>
+  </si>
+  <si>
     <t>01/04/2026 até 30/04/2026</t>
-  </si>
-  <si>
-    <t>Data de Criação do Orçamento</t>
-  </si>
-  <si>
-    <t>/  /     00:00 até   /  /     00:00</t>
-  </si>
-  <si>
-    <t>Data de Criação do Contrato</t>
-  </si>
-  <si>
-    <t>/  /     até   /  /</t>
-  </si>
-  <si>
-    <t>Data de Assinatura do Contrato</t>
   </si>
   <si>
     <t>Data de Criação do Cliente</t>
@@ -512,15 +512,15 @@
         <v>23</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B19" s="3" t="s">
         <v>25</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="20">
@@ -528,7 +528,7 @@
         <v>26</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
     </row>
     <row r="21">
@@ -536,7 +536,7 @@
         <v>27</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
     </row>
     <row r="22">

</xml_diff>